<commit_message>
Create new django command
</commit_message>
<xml_diff>
--- a/Census/utils/project.xlsx
+++ b/Census/utils/project.xlsx
@@ -129,7 +129,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="651">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="652">
   <si>
     <t>Ecosystème Tech Togo</t>
   </si>
@@ -1764,9 +1764,6 @@
     <t>https://woelab.hubcity.africa</t>
   </si>
   <si>
-    <t>https://numerique.gouv.tg/</t>
-  </si>
-  <si>
     <t>Established in August 2012, WoeLab is Togo's first open-source laboratory for social and technological innovation. It was founded as part of the "Lomé HubCité africaine" urban utopia developed by the platform L’Africaine d’Architecture and its creator, Sénamé Koffi Agbodjinou.
 HubCité is an alternative and participatory urban planning project. It challenges traditional regulatory and elitist approaches by proposing a model where citizens themselves take charge of their neighborhood's destiny. This is achieved through the installation of a network of local tech hubs within a given territory. These hubs are easily replicable, open to all, and designed to promote a culture of sharing while incubating #LowHighTech—technology accessible enough to permeate the most modest layers of the population. By engaging with these spaces, everyday people regain the drive for collective action, eventually reclaiming the capacity to think, design, and build the city of tomorrow themselves.
 The ambition is to rethink the African city around these centers of innovation and have it "manufactured" by the businesses that emerge from them. The 11 collaborative startups created and incubated at WoeLab under the SiliconVilla program are built on the intuition that the entrepreneur is destined to replace the architect, the urban planner, or the policymaker in the production of the city. Each startup works on a specific urban theme, such as waste management, mobility, or resource allocation.
@@ -2099,6 +2096,12 @@
   </si>
   <si>
     <t>Flutter TG</t>
+  </si>
+  <si>
+    <t>Node.js, Express.js</t>
+  </si>
+  <si>
+    <t>https://djantatechhub.gouv.tg/</t>
   </si>
 </sst>
 </file>
@@ -2295,6 +2298,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2302,13 +2311,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2596,18 +2599,18 @@
       <c r="A1" s="1"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
       <c r="P1" s="2"/>
@@ -2664,18 +2667,18 @@
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
-      <c r="D3" s="25" t="s">
-        <v>545</v>
-      </c>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24"/>
+      <c r="D3" s="27" t="s">
+        <v>544</v>
+      </c>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="26"/>
+      <c r="K3" s="26"/>
+      <c r="L3" s="26"/>
+      <c r="M3" s="26"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
@@ -2721,7 +2724,7 @@
         <v>4</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="L4" s="7" t="s">
         <v>538</v>
@@ -2756,7 +2759,7 @@
         <v>6</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F5" s="12" t="s">
         <v>7</v>
@@ -2774,7 +2777,7 @@
         <v>11</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="L5" s="12" t="s">
         <v>12</v>
@@ -2806,7 +2809,7 @@
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="1" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="E6" s="11" t="s">
         <v>14</v>
@@ -2827,7 +2830,7 @@
         <v>11</v>
       </c>
       <c r="K6" s="12" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="L6" s="12" t="s">
         <v>17</v>
@@ -2880,13 +2883,13 @@
         <v>11</v>
       </c>
       <c r="K7" s="12" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="L7" s="12" t="s">
         <v>23</v>
       </c>
       <c r="M7" s="20" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -2933,7 +2936,7 @@
         <v>11</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="L8" s="12" t="s">
         <v>28</v>
@@ -2986,7 +2989,7 @@
         <v>11</v>
       </c>
       <c r="K9" s="12" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="L9" s="12" t="s">
         <v>36</v>
@@ -3039,7 +3042,7 @@
         <v>30</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L10" s="12" t="s">
         <v>42</v>
@@ -3092,7 +3095,7 @@
         <v>30</v>
       </c>
       <c r="K11" s="12" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="L11" s="12" t="s">
         <v>49</v>
@@ -3162,18 +3165,18 @@
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="27" t="s">
-        <v>546</v>
-      </c>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="27"/>
-      <c r="J13" s="27"/>
-      <c r="K13" s="27"/>
-      <c r="L13" s="27"/>
-      <c r="M13" s="27"/>
+      <c r="D13" s="28" t="s">
+        <v>545</v>
+      </c>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="28"/>
+      <c r="K13" s="28"/>
+      <c r="L13" s="28"/>
+      <c r="M13" s="28"/>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
       <c r="P13" s="2"/>
@@ -3219,7 +3222,7 @@
         <v>11</v>
       </c>
       <c r="K14" s="12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L14" s="12" t="s">
         <v>57</v>
@@ -3272,7 +3275,7 @@
         <v>30</v>
       </c>
       <c r="K15" s="12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L15" s="12" t="s">
         <v>63</v>
@@ -3325,7 +3328,7 @@
         <v>30</v>
       </c>
       <c r="K16" s="12" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="L16" s="12" t="s">
         <v>69</v>
@@ -3378,7 +3381,7 @@
         <v>77</v>
       </c>
       <c r="K17" s="12" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="L17" s="12" t="s">
         <v>78</v>
@@ -3431,7 +3434,7 @@
         <v>77</v>
       </c>
       <c r="K18" s="12" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="L18" s="12" t="s">
         <v>85</v>
@@ -3463,7 +3466,7 @@
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>87</v>
@@ -3484,7 +3487,7 @@
         <v>77</v>
       </c>
       <c r="K19" s="12" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="L19" s="12" t="s">
         <v>92</v>
@@ -3554,18 +3557,18 @@
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
-      <c r="D21" s="26" t="s">
-        <v>547</v>
-      </c>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="26"/>
-      <c r="I21" s="26"/>
-      <c r="J21" s="26"/>
-      <c r="K21" s="26"/>
-      <c r="L21" s="26"/>
-      <c r="M21" s="26"/>
+      <c r="D21" s="23" t="s">
+        <v>546</v>
+      </c>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="23"/>
+      <c r="K21" s="23"/>
+      <c r="L21" s="23"/>
+      <c r="M21" s="23"/>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
       <c r="P21" s="2"/>
@@ -3611,7 +3614,7 @@
         <v>98</v>
       </c>
       <c r="K22" s="12" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="L22" s="12" t="s">
         <v>99</v>
@@ -3664,7 +3667,7 @@
         <v>11</v>
       </c>
       <c r="K23" s="12" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="L23" s="12" t="s">
         <v>105</v>
@@ -3717,7 +3720,7 @@
         <v>30</v>
       </c>
       <c r="K24" s="12" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="L24" s="12" t="s">
         <v>111</v>
@@ -3770,7 +3773,7 @@
         <v>30</v>
       </c>
       <c r="K25" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L25" s="12" t="s">
         <v>117</v>
@@ -3823,7 +3826,7 @@
         <v>30</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="L26" s="12" t="s">
         <v>123</v>
@@ -3876,7 +3879,7 @@
         <v>77</v>
       </c>
       <c r="K27" s="12" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="L27" s="12" t="s">
         <v>129</v>
@@ -3946,18 +3949,18 @@
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
-      <c r="D29" s="26" t="s">
+      <c r="D29" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26"/>
-      <c r="H29" s="26"/>
-      <c r="I29" s="26"/>
-      <c r="J29" s="26"/>
-      <c r="K29" s="26"/>
-      <c r="L29" s="26"/>
-      <c r="M29" s="26"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="23"/>
+      <c r="I29" s="23"/>
+      <c r="J29" s="23"/>
+      <c r="K29" s="23"/>
+      <c r="L29" s="23"/>
+      <c r="M29" s="23"/>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
       <c r="P29" s="2"/>
@@ -3977,7 +3980,7 @@
       <c r="AD29" s="2"/>
       <c r="AE29" s="2"/>
     </row>
-    <row r="30" spans="1:31" ht="105">
+    <row r="30" spans="1:31" ht="120">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -4003,7 +4006,7 @@
         <v>30</v>
       </c>
       <c r="K30" s="12" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="L30" s="12" t="s">
         <v>136</v>
@@ -4056,7 +4059,7 @@
         <v>30</v>
       </c>
       <c r="K31" s="12" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="L31" s="12" t="s">
         <v>142</v>
@@ -4109,7 +4112,7 @@
         <v>77</v>
       </c>
       <c r="K32" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L32" s="12" t="s">
         <v>148</v>
@@ -4162,7 +4165,7 @@
         <v>30</v>
       </c>
       <c r="K33" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L33" s="12" t="s">
         <v>154</v>
@@ -4232,18 +4235,18 @@
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
-      <c r="D35" s="26" t="s">
-        <v>548</v>
-      </c>
-      <c r="E35" s="26"/>
-      <c r="F35" s="26"/>
-      <c r="G35" s="26"/>
-      <c r="H35" s="26"/>
-      <c r="I35" s="26"/>
-      <c r="J35" s="26"/>
-      <c r="K35" s="26"/>
-      <c r="L35" s="26"/>
-      <c r="M35" s="26"/>
+      <c r="D35" s="23" t="s">
+        <v>547</v>
+      </c>
+      <c r="E35" s="23"/>
+      <c r="F35" s="23"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="23"/>
+      <c r="I35" s="23"/>
+      <c r="J35" s="23"/>
+      <c r="K35" s="23"/>
+      <c r="L35" s="23"/>
+      <c r="M35" s="23"/>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" s="2"/>
@@ -4289,7 +4292,7 @@
         <v>11</v>
       </c>
       <c r="K36" s="12" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="L36" s="12" t="s">
         <v>160</v>
@@ -4342,7 +4345,7 @@
         <v>11</v>
       </c>
       <c r="K37" s="12" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="L37" s="12" t="s">
         <v>166</v>
@@ -4395,7 +4398,7 @@
         <v>30</v>
       </c>
       <c r="K38" s="12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L38" s="12" t="s">
         <v>172</v>
@@ -4448,7 +4451,7 @@
         <v>30</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="L39" s="12" t="s">
         <v>180</v>
@@ -4479,13 +4482,13 @@
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="E40" s="9" t="s">
         <v>602</v>
       </c>
-      <c r="E40" s="9" t="s">
+      <c r="F40" s="12" t="s">
         <v>603</v>
-      </c>
-      <c r="F40" s="12" t="s">
-        <v>604</v>
       </c>
       <c r="G40" s="12" t="s">
         <v>177</v>
@@ -4494,19 +4497,19 @@
         <v>178</v>
       </c>
       <c r="I40" s="12" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="J40" s="12" t="s">
         <v>77</v>
       </c>
       <c r="K40" s="12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L40" s="12" t="s">
+        <v>605</v>
+      </c>
+      <c r="M40" s="20" t="s">
         <v>606</v>
-      </c>
-      <c r="M40" s="20" t="s">
-        <v>607</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -4548,18 +4551,18 @@
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
-      <c r="D42" s="26" t="s">
-        <v>549</v>
-      </c>
-      <c r="E42" s="26"/>
-      <c r="F42" s="26"/>
-      <c r="G42" s="26"/>
-      <c r="H42" s="26"/>
-      <c r="I42" s="26"/>
-      <c r="J42" s="26"/>
-      <c r="K42" s="26"/>
-      <c r="L42" s="26"/>
-      <c r="M42" s="26"/>
+      <c r="D42" s="23" t="s">
+        <v>548</v>
+      </c>
+      <c r="E42" s="23"/>
+      <c r="F42" s="23"/>
+      <c r="G42" s="23"/>
+      <c r="H42" s="23"/>
+      <c r="I42" s="23"/>
+      <c r="J42" s="23"/>
+      <c r="K42" s="23"/>
+      <c r="L42" s="23"/>
+      <c r="M42" s="23"/>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
       <c r="P42" s="2"/>
@@ -4605,7 +4608,7 @@
         <v>11</v>
       </c>
       <c r="K43" s="12" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="L43" s="12" t="s">
         <v>186</v>
@@ -4658,7 +4661,7 @@
         <v>11</v>
       </c>
       <c r="K44" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L44" s="12" t="s">
         <v>192</v>
@@ -4711,7 +4714,7 @@
         <v>30</v>
       </c>
       <c r="K45" s="12" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="L45" s="12" t="s">
         <v>198</v>
@@ -4738,7 +4741,7 @@
       <c r="AD45" s="2"/>
       <c r="AE45" s="2"/>
     </row>
-    <row r="46" spans="1:31" ht="105">
+    <row r="46" spans="1:31" ht="120">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -4764,7 +4767,7 @@
         <v>30</v>
       </c>
       <c r="K46" s="12" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="L46" s="12" t="s">
         <v>205</v>
@@ -4817,7 +4820,7 @@
         <v>30</v>
       </c>
       <c r="K47" s="12" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="L47" s="12" t="s">
         <v>211</v>
@@ -4870,7 +4873,7 @@
         <v>77</v>
       </c>
       <c r="K48" s="12" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="L48" s="12" t="s">
         <v>218</v>
@@ -4902,7 +4905,7 @@
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="1" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>220</v>
@@ -4923,7 +4926,7 @@
         <v>11</v>
       </c>
       <c r="K49" s="12" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="L49" s="12" t="s">
         <v>224</v>
@@ -4995,18 +4998,18 @@
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
-      <c r="D51" s="26" t="s">
+      <c r="D51" s="23" t="s">
         <v>226</v>
       </c>
-      <c r="E51" s="26"/>
-      <c r="F51" s="26"/>
-      <c r="G51" s="26"/>
-      <c r="H51" s="26"/>
-      <c r="I51" s="26"/>
-      <c r="J51" s="26"/>
-      <c r="K51" s="26"/>
-      <c r="L51" s="26"/>
-      <c r="M51" s="26"/>
+      <c r="E51" s="23"/>
+      <c r="F51" s="23"/>
+      <c r="G51" s="23"/>
+      <c r="H51" s="23"/>
+      <c r="I51" s="23"/>
+      <c r="J51" s="23"/>
+      <c r="K51" s="23"/>
+      <c r="L51" s="23"/>
+      <c r="M51" s="23"/>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
       <c r="P51" s="2"/>
@@ -5052,7 +5055,7 @@
         <v>11</v>
       </c>
       <c r="K52" s="12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L52" s="12" t="s">
         <v>231</v>
@@ -5084,7 +5087,7 @@
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
       <c r="D53" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>233</v>
@@ -5105,7 +5108,7 @@
         <v>98</v>
       </c>
       <c r="K53" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L53" s="12" t="s">
         <v>236</v>
@@ -5158,7 +5161,7 @@
         <v>30</v>
       </c>
       <c r="K54" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L54" s="12" t="s">
         <v>243</v>
@@ -5185,7 +5188,7 @@
       <c r="AD54" s="2"/>
       <c r="AE54" s="2"/>
     </row>
-    <row r="55" spans="1:31" ht="105">
+    <row r="55" spans="1:31" ht="120">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -5211,7 +5214,7 @@
         <v>30</v>
       </c>
       <c r="K55" s="12" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="L55" s="12" t="s">
         <v>249</v>
@@ -5264,7 +5267,7 @@
         <v>30</v>
       </c>
       <c r="K56" s="12" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="L56" s="12" t="s">
         <v>255</v>
@@ -5317,7 +5320,7 @@
         <v>30</v>
       </c>
       <c r="K57" s="12" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="L57" s="12" t="s">
         <v>262</v>
@@ -5389,18 +5392,18 @@
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
-      <c r="D59" s="26" t="s">
-        <v>550</v>
-      </c>
-      <c r="E59" s="26"/>
-      <c r="F59" s="26"/>
-      <c r="G59" s="26"/>
-      <c r="H59" s="26"/>
-      <c r="I59" s="26"/>
-      <c r="J59" s="26"/>
-      <c r="K59" s="26"/>
-      <c r="L59" s="26"/>
-      <c r="M59" s="26"/>
+      <c r="D59" s="23" t="s">
+        <v>549</v>
+      </c>
+      <c r="E59" s="23"/>
+      <c r="F59" s="23"/>
+      <c r="G59" s="23"/>
+      <c r="H59" s="23"/>
+      <c r="I59" s="23"/>
+      <c r="J59" s="23"/>
+      <c r="K59" s="23"/>
+      <c r="L59" s="23"/>
+      <c r="M59" s="23"/>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
       <c r="P59" s="2"/>
@@ -5446,7 +5449,7 @@
         <v>30</v>
       </c>
       <c r="K60" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L60" s="12" t="s">
         <v>268</v>
@@ -5499,7 +5502,7 @@
         <v>77</v>
       </c>
       <c r="K61" s="12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L61" s="12" t="s">
         <v>274</v>
@@ -5552,7 +5555,7 @@
         <v>30</v>
       </c>
       <c r="K62" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L62" s="12" t="s">
         <v>280</v>
@@ -5590,13 +5593,13 @@
         <v>283</v>
       </c>
       <c r="F63" s="12" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="G63" s="12" t="s">
         <v>284</v>
       </c>
       <c r="H63" s="12" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="I63" s="12" t="s">
         <v>285</v>
@@ -5605,7 +5608,7 @@
         <v>30</v>
       </c>
       <c r="K63" s="12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L63" s="12" t="s">
         <v>10</v>
@@ -5677,18 +5680,18 @@
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
-      <c r="D65" s="26" t="s">
-        <v>551</v>
-      </c>
-      <c r="E65" s="26"/>
-      <c r="F65" s="26"/>
-      <c r="G65" s="26"/>
-      <c r="H65" s="26"/>
-      <c r="I65" s="26"/>
-      <c r="J65" s="26"/>
-      <c r="K65" s="26"/>
-      <c r="L65" s="26"/>
-      <c r="M65" s="26"/>
+      <c r="D65" s="23" t="s">
+        <v>550</v>
+      </c>
+      <c r="E65" s="23"/>
+      <c r="F65" s="23"/>
+      <c r="G65" s="23"/>
+      <c r="H65" s="23"/>
+      <c r="I65" s="23"/>
+      <c r="J65" s="23"/>
+      <c r="K65" s="23"/>
+      <c r="L65" s="23"/>
+      <c r="M65" s="23"/>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
       <c r="P65" s="2"/>
@@ -5734,7 +5737,7 @@
         <v>11</v>
       </c>
       <c r="K66" s="12" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="L66" s="12" t="s">
         <v>290</v>
@@ -5787,7 +5790,7 @@
         <v>30</v>
       </c>
       <c r="K67" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L67" s="12" t="s">
         <v>296</v>
@@ -5840,7 +5843,7 @@
         <v>11</v>
       </c>
       <c r="K68" s="12" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="L68" s="12" t="s">
         <v>302</v>
@@ -5893,7 +5896,7 @@
         <v>11</v>
       </c>
       <c r="K69" s="12" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="L69" s="12" t="s">
         <v>308</v>
@@ -5946,7 +5949,7 @@
         <v>30</v>
       </c>
       <c r="K70" s="12" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="L70" s="12" t="s">
         <v>314</v>
@@ -6018,18 +6021,18 @@
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
-      <c r="D72" s="26" t="s">
-        <v>552</v>
-      </c>
-      <c r="E72" s="26"/>
-      <c r="F72" s="26"/>
-      <c r="G72" s="26"/>
-      <c r="H72" s="26"/>
-      <c r="I72" s="26"/>
-      <c r="J72" s="26"/>
-      <c r="K72" s="26"/>
-      <c r="L72" s="26"/>
-      <c r="M72" s="26"/>
+      <c r="D72" s="23" t="s">
+        <v>551</v>
+      </c>
+      <c r="E72" s="23"/>
+      <c r="F72" s="23"/>
+      <c r="G72" s="23"/>
+      <c r="H72" s="23"/>
+      <c r="I72" s="23"/>
+      <c r="J72" s="23"/>
+      <c r="K72" s="23"/>
+      <c r="L72" s="23"/>
+      <c r="M72" s="23"/>
       <c r="N72" s="2"/>
       <c r="O72" s="2"/>
       <c r="P72" s="2"/>
@@ -6075,7 +6078,7 @@
         <v>11</v>
       </c>
       <c r="K73" s="12" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="L73" s="12" t="s">
         <v>320</v>
@@ -6146,18 +6149,18 @@
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
-      <c r="D75" s="28" t="s">
+      <c r="D75" s="24" t="s">
         <v>322</v>
       </c>
-      <c r="E75" s="28"/>
-      <c r="F75" s="28"/>
-      <c r="G75" s="28"/>
-      <c r="H75" s="28"/>
-      <c r="I75" s="28"/>
-      <c r="J75" s="28"/>
-      <c r="K75" s="28"/>
-      <c r="L75" s="28"/>
-      <c r="M75" s="28"/>
+      <c r="E75" s="24"/>
+      <c r="F75" s="24"/>
+      <c r="G75" s="24"/>
+      <c r="H75" s="24"/>
+      <c r="I75" s="24"/>
+      <c r="J75" s="24"/>
+      <c r="K75" s="24"/>
+      <c r="L75" s="24"/>
+      <c r="M75" s="24"/>
       <c r="N75" s="2"/>
       <c r="O75" s="2"/>
       <c r="P75" s="2"/>
@@ -6222,18 +6225,18 @@
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
-      <c r="D77" s="26" t="s">
+      <c r="D77" s="23" t="s">
         <v>323</v>
       </c>
-      <c r="E77" s="26"/>
-      <c r="F77" s="26"/>
-      <c r="G77" s="26"/>
-      <c r="H77" s="26"/>
-      <c r="I77" s="26"/>
-      <c r="J77" s="26"/>
-      <c r="K77" s="26"/>
-      <c r="L77" s="26"/>
-      <c r="M77" s="26"/>
+      <c r="E77" s="23"/>
+      <c r="F77" s="23"/>
+      <c r="G77" s="23"/>
+      <c r="H77" s="23"/>
+      <c r="I77" s="23"/>
+      <c r="J77" s="23"/>
+      <c r="K77" s="23"/>
+      <c r="L77" s="23"/>
+      <c r="M77" s="23"/>
       <c r="N77" s="2"/>
       <c r="O77" s="2"/>
       <c r="P77" s="2"/>
@@ -6279,7 +6282,7 @@
         <v>30</v>
       </c>
       <c r="K78" s="12" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="L78" s="12" t="s">
         <v>329</v>
@@ -6332,7 +6335,7 @@
         <v>30</v>
       </c>
       <c r="K79" s="12" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="L79" s="12" t="s">
         <v>335</v>
@@ -6404,18 +6407,18 @@
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
-      <c r="D81" s="26" t="s">
-        <v>553</v>
-      </c>
-      <c r="E81" s="26"/>
-      <c r="F81" s="26"/>
-      <c r="G81" s="26"/>
-      <c r="H81" s="26"/>
-      <c r="I81" s="26"/>
-      <c r="J81" s="26"/>
-      <c r="K81" s="26"/>
-      <c r="L81" s="26"/>
-      <c r="M81" s="26"/>
+      <c r="D81" s="23" t="s">
+        <v>552</v>
+      </c>
+      <c r="E81" s="23"/>
+      <c r="F81" s="23"/>
+      <c r="G81" s="23"/>
+      <c r="H81" s="23"/>
+      <c r="I81" s="23"/>
+      <c r="J81" s="23"/>
+      <c r="K81" s="23"/>
+      <c r="L81" s="23"/>
+      <c r="M81" s="23"/>
       <c r="N81" s="2"/>
       <c r="O81" s="2"/>
       <c r="P81" s="2"/>
@@ -6461,7 +6464,7 @@
         <v>30</v>
       </c>
       <c r="K82" s="12" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="L82" s="12" t="s">
         <v>342</v>
@@ -6514,7 +6517,7 @@
         <v>30</v>
       </c>
       <c r="K83" s="12" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="L83" s="12" t="s">
         <v>348</v>
@@ -6586,18 +6589,18 @@
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
-      <c r="D85" s="26" t="s">
-        <v>554</v>
-      </c>
-      <c r="E85" s="26"/>
-      <c r="F85" s="26"/>
-      <c r="G85" s="26"/>
-      <c r="H85" s="26"/>
-      <c r="I85" s="26"/>
-      <c r="J85" s="26"/>
-      <c r="K85" s="26"/>
-      <c r="L85" s="26"/>
-      <c r="M85" s="26"/>
+      <c r="D85" s="23" t="s">
+        <v>553</v>
+      </c>
+      <c r="E85" s="23"/>
+      <c r="F85" s="23"/>
+      <c r="G85" s="23"/>
+      <c r="H85" s="23"/>
+      <c r="I85" s="23"/>
+      <c r="J85" s="23"/>
+      <c r="K85" s="23"/>
+      <c r="L85" s="23"/>
+      <c r="M85" s="23"/>
       <c r="N85" s="2"/>
       <c r="O85" s="2"/>
       <c r="P85" s="2"/>
@@ -6643,7 +6646,7 @@
         <v>30</v>
       </c>
       <c r="K86" s="12" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="L86" s="12" t="s">
         <v>353</v>
@@ -6696,7 +6699,7 @@
         <v>30</v>
       </c>
       <c r="K87" s="12" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="L87" s="12" t="s">
         <v>360</v>
@@ -6728,7 +6731,7 @@
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="1" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="E88" s="9" t="s">
         <v>362</v>
@@ -6749,7 +6752,7 @@
         <v>30</v>
       </c>
       <c r="K88" s="12" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="L88" s="12" t="s">
         <v>364</v>
@@ -6802,7 +6805,7 @@
         <v>30</v>
       </c>
       <c r="K89" s="12" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="L89" s="12" t="s">
         <v>369</v>
@@ -6834,7 +6837,7 @@
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="1" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="E90" s="9" t="s">
         <v>371</v>
@@ -6855,7 +6858,7 @@
         <v>30</v>
       </c>
       <c r="K90" s="12" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="L90" s="12" t="s">
         <v>348</v>
@@ -6927,18 +6930,18 @@
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
-      <c r="D92" s="26" t="s">
+      <c r="D92" s="23" t="s">
         <v>375</v>
       </c>
-      <c r="E92" s="26"/>
-      <c r="F92" s="26"/>
-      <c r="G92" s="26"/>
-      <c r="H92" s="26"/>
-      <c r="I92" s="26"/>
-      <c r="J92" s="26"/>
-      <c r="K92" s="26"/>
-      <c r="L92" s="26"/>
-      <c r="M92" s="26"/>
+      <c r="E92" s="23"/>
+      <c r="F92" s="23"/>
+      <c r="G92" s="23"/>
+      <c r="H92" s="23"/>
+      <c r="I92" s="23"/>
+      <c r="J92" s="23"/>
+      <c r="K92" s="23"/>
+      <c r="L92" s="23"/>
+      <c r="M92" s="23"/>
       <c r="N92" s="2"/>
       <c r="O92" s="2"/>
       <c r="P92" s="2"/>
@@ -6984,7 +6987,7 @@
         <v>30</v>
       </c>
       <c r="K93" s="12" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="L93" s="12" t="s">
         <v>379</v>
@@ -7037,7 +7040,7 @@
         <v>30</v>
       </c>
       <c r="K94" s="12" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="L94" s="12" t="s">
         <v>385</v>
@@ -7090,7 +7093,7 @@
         <v>30</v>
       </c>
       <c r="K95" s="12" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="L95" s="12" t="s">
         <v>390</v>
@@ -7143,7 +7146,7 @@
         <v>30</v>
       </c>
       <c r="K96" s="12" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="L96" s="12" t="s">
         <v>396</v>
@@ -7215,18 +7218,18 @@
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
-      <c r="D98" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="E98" s="26"/>
-      <c r="F98" s="26"/>
-      <c r="G98" s="26"/>
-      <c r="H98" s="26"/>
-      <c r="I98" s="26"/>
-      <c r="J98" s="26"/>
-      <c r="K98" s="26"/>
-      <c r="L98" s="26"/>
-      <c r="M98" s="26"/>
+      <c r="D98" s="23" t="s">
+        <v>554</v>
+      </c>
+      <c r="E98" s="23"/>
+      <c r="F98" s="23"/>
+      <c r="G98" s="23"/>
+      <c r="H98" s="23"/>
+      <c r="I98" s="23"/>
+      <c r="J98" s="23"/>
+      <c r="K98" s="23"/>
+      <c r="L98" s="23"/>
+      <c r="M98" s="23"/>
       <c r="N98" s="2"/>
       <c r="O98" s="2"/>
       <c r="P98" s="2"/>
@@ -7272,7 +7275,7 @@
         <v>77</v>
       </c>
       <c r="K99" s="12" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="L99" s="12" t="s">
         <v>402</v>
@@ -7304,13 +7307,13 @@
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
       <c r="D100" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="E100" s="9" t="s">
+        <v>584</v>
+      </c>
+      <c r="F100" s="12" t="s">
         <v>583</v>
-      </c>
-      <c r="E100" s="9" t="s">
-        <v>585</v>
-      </c>
-      <c r="F100" s="12" t="s">
-        <v>584</v>
       </c>
       <c r="G100" s="12" t="s">
         <v>177</v>
@@ -7319,19 +7322,19 @@
         <v>9</v>
       </c>
       <c r="I100" s="12" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="J100" s="12" t="s">
         <v>77</v>
       </c>
       <c r="K100" s="12" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="L100" s="12" t="s">
+        <v>587</v>
+      </c>
+      <c r="M100" s="10" t="s">
         <v>588</v>
-      </c>
-      <c r="M100" s="10" t="s">
-        <v>589</v>
       </c>
       <c r="N100" s="2"/>
       <c r="O100" s="2"/>
@@ -7397,18 +7400,18 @@
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
       <c r="C102" s="2"/>
-      <c r="D102" s="26" t="s">
-        <v>556</v>
-      </c>
-      <c r="E102" s="26"/>
-      <c r="F102" s="26"/>
-      <c r="G102" s="26"/>
-      <c r="H102" s="26"/>
-      <c r="I102" s="26"/>
-      <c r="J102" s="26"/>
-      <c r="K102" s="26"/>
-      <c r="L102" s="26"/>
-      <c r="M102" s="26"/>
+      <c r="D102" s="23" t="s">
+        <v>555</v>
+      </c>
+      <c r="E102" s="23"/>
+      <c r="F102" s="23"/>
+      <c r="G102" s="23"/>
+      <c r="H102" s="23"/>
+      <c r="I102" s="23"/>
+      <c r="J102" s="23"/>
+      <c r="K102" s="23"/>
+      <c r="L102" s="23"/>
+      <c r="M102" s="23"/>
       <c r="N102" s="2"/>
       <c r="O102" s="2"/>
       <c r="P102" s="2"/>
@@ -7454,7 +7457,7 @@
         <v>77</v>
       </c>
       <c r="K103" s="12" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="L103" s="12" t="s">
         <v>407</v>
@@ -7507,7 +7510,7 @@
         <v>77</v>
       </c>
       <c r="K104" s="12" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="L104" s="12" t="s">
         <v>412</v>
@@ -7560,7 +7563,7 @@
         <v>77</v>
       </c>
       <c r="K105" s="12" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="L105" s="12" t="s">
         <v>417</v>
@@ -7613,7 +7616,7 @@
         <v>77</v>
       </c>
       <c r="K106" s="12" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="L106" s="12" t="s">
         <v>422</v>
@@ -7666,7 +7669,7 @@
         <v>77</v>
       </c>
       <c r="K107" s="12" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="L107" s="12" t="s">
         <v>428</v>
@@ -7719,7 +7722,7 @@
         <v>77</v>
       </c>
       <c r="K108" s="12" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="L108" s="12" t="s">
         <v>417</v>
@@ -7791,18 +7794,18 @@
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
-      <c r="D110" s="26" t="s">
+      <c r="D110" s="23" t="s">
         <v>435</v>
       </c>
-      <c r="E110" s="26"/>
-      <c r="F110" s="26"/>
-      <c r="G110" s="26"/>
-      <c r="H110" s="26"/>
-      <c r="I110" s="26"/>
-      <c r="J110" s="26"/>
-      <c r="K110" s="26"/>
-      <c r="L110" s="26"/>
-      <c r="M110" s="26"/>
+      <c r="E110" s="23"/>
+      <c r="F110" s="23"/>
+      <c r="G110" s="23"/>
+      <c r="H110" s="23"/>
+      <c r="I110" s="23"/>
+      <c r="J110" s="23"/>
+      <c r="K110" s="23"/>
+      <c r="L110" s="23"/>
+      <c r="M110" s="23"/>
       <c r="N110" s="2"/>
       <c r="O110" s="2"/>
       <c r="P110" s="2"/>
@@ -7827,7 +7830,7 @@
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
       <c r="D111" s="1" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="E111" s="9" t="s">
         <v>436</v>
@@ -7848,7 +7851,7 @@
         <v>77</v>
       </c>
       <c r="K111" s="12" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="L111" s="12" t="s">
         <v>439</v>
@@ -7901,7 +7904,7 @@
         <v>77</v>
       </c>
       <c r="K112" s="12" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="L112" s="12" t="s">
         <v>445</v>
@@ -7973,18 +7976,18 @@
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
-      <c r="D114" s="26" t="s">
-        <v>600</v>
-      </c>
-      <c r="E114" s="26"/>
-      <c r="F114" s="26"/>
-      <c r="G114" s="26"/>
-      <c r="H114" s="26"/>
-      <c r="I114" s="26"/>
-      <c r="J114" s="26"/>
-      <c r="K114" s="26"/>
-      <c r="L114" s="26"/>
-      <c r="M114" s="26"/>
+      <c r="D114" s="23" t="s">
+        <v>599</v>
+      </c>
+      <c r="E114" s="23"/>
+      <c r="F114" s="23"/>
+      <c r="G114" s="23"/>
+      <c r="H114" s="23"/>
+      <c r="I114" s="23"/>
+      <c r="J114" s="23"/>
+      <c r="K114" s="23"/>
+      <c r="L114" s="23"/>
+      <c r="M114" s="23"/>
       <c r="N114" s="2"/>
       <c r="O114" s="2"/>
       <c r="P114" s="2"/>
@@ -8030,7 +8033,7 @@
         <v>77</v>
       </c>
       <c r="K115" s="12" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="L115" s="12" t="s">
         <v>379</v>
@@ -8083,7 +8086,7 @@
         <v>77</v>
       </c>
       <c r="K116" s="12" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="L116" s="12" t="s">
         <v>464</v>
@@ -8136,7 +8139,7 @@
         <v>77</v>
       </c>
       <c r="K117" s="12" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="L117" s="12" t="s">
         <v>464</v>
@@ -8208,18 +8211,18 @@
       <c r="A119" s="2"/>
       <c r="B119" s="2"/>
       <c r="C119" s="2"/>
-      <c r="D119" s="26" t="s">
-        <v>557</v>
-      </c>
-      <c r="E119" s="26"/>
-      <c r="F119" s="26"/>
-      <c r="G119" s="26"/>
-      <c r="H119" s="26"/>
-      <c r="I119" s="26"/>
-      <c r="J119" s="26"/>
-      <c r="K119" s="26"/>
-      <c r="L119" s="26"/>
-      <c r="M119" s="26"/>
+      <c r="D119" s="23" t="s">
+        <v>556</v>
+      </c>
+      <c r="E119" s="23"/>
+      <c r="F119" s="23"/>
+      <c r="G119" s="23"/>
+      <c r="H119" s="23"/>
+      <c r="I119" s="23"/>
+      <c r="J119" s="23"/>
+      <c r="K119" s="23"/>
+      <c r="L119" s="23"/>
+      <c r="M119" s="23"/>
       <c r="N119" s="2"/>
       <c r="O119" s="2"/>
       <c r="P119" s="2"/>
@@ -8244,7 +8247,7 @@
       <c r="B120" s="2"/>
       <c r="C120" s="2"/>
       <c r="D120" s="1" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="E120" s="9" t="s">
         <v>469</v>
@@ -8265,7 +8268,7 @@
         <v>77</v>
       </c>
       <c r="K120" s="12" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="L120" s="12" t="s">
         <v>348</v>
@@ -8318,7 +8321,7 @@
         <v>77</v>
       </c>
       <c r="K121" s="12" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="L121" s="12" t="s">
         <v>477</v>
@@ -8390,18 +8393,18 @@
       <c r="A123" s="2"/>
       <c r="B123" s="2"/>
       <c r="C123" s="2"/>
-      <c r="D123" s="26" t="s">
+      <c r="D123" s="23" t="s">
         <v>479</v>
       </c>
-      <c r="E123" s="26"/>
-      <c r="F123" s="26"/>
-      <c r="G123" s="26"/>
-      <c r="H123" s="26"/>
-      <c r="I123" s="26"/>
-      <c r="J123" s="26"/>
-      <c r="K123" s="26"/>
-      <c r="L123" s="26"/>
-      <c r="M123" s="26"/>
+      <c r="E123" s="23"/>
+      <c r="F123" s="23"/>
+      <c r="G123" s="23"/>
+      <c r="H123" s="23"/>
+      <c r="I123" s="23"/>
+      <c r="J123" s="23"/>
+      <c r="K123" s="23"/>
+      <c r="L123" s="23"/>
+      <c r="M123" s="23"/>
       <c r="N123" s="2"/>
       <c r="O123" s="2"/>
       <c r="P123" s="2"/>
@@ -8447,7 +8450,7 @@
         <v>77</v>
       </c>
       <c r="K124" s="12" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="L124" s="12" t="s">
         <v>484</v>
@@ -8519,18 +8522,18 @@
       <c r="A126" s="2"/>
       <c r="B126" s="2"/>
       <c r="C126" s="2"/>
-      <c r="D126" s="26" t="s">
-        <v>558</v>
-      </c>
-      <c r="E126" s="26"/>
-      <c r="F126" s="26"/>
-      <c r="G126" s="26"/>
-      <c r="H126" s="26"/>
-      <c r="I126" s="26"/>
-      <c r="J126" s="26"/>
-      <c r="K126" s="26"/>
-      <c r="L126" s="26"/>
-      <c r="M126" s="26"/>
+      <c r="D126" s="23" t="s">
+        <v>557</v>
+      </c>
+      <c r="E126" s="23"/>
+      <c r="F126" s="23"/>
+      <c r="G126" s="23"/>
+      <c r="H126" s="23"/>
+      <c r="I126" s="23"/>
+      <c r="J126" s="23"/>
+      <c r="K126" s="23"/>
+      <c r="L126" s="23"/>
+      <c r="M126" s="23"/>
       <c r="N126" s="2"/>
       <c r="O126" s="2"/>
       <c r="P126" s="2"/>
@@ -8576,7 +8579,7 @@
         <v>77</v>
       </c>
       <c r="K127" s="12" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="L127" s="12" t="s">
         <v>452</v>
@@ -8608,13 +8611,13 @@
       <c r="B128" s="2"/>
       <c r="C128" s="2"/>
       <c r="D128" s="1" t="s">
+        <v>608</v>
+      </c>
+      <c r="E128" s="9" t="s">
+        <v>611</v>
+      </c>
+      <c r="F128" s="12" t="s">
         <v>609</v>
-      </c>
-      <c r="E128" s="9" t="s">
-        <v>612</v>
-      </c>
-      <c r="F128" s="12" t="s">
-        <v>610</v>
       </c>
       <c r="G128" s="12" t="s">
         <v>340</v>
@@ -8629,13 +8632,13 @@
         <v>30</v>
       </c>
       <c r="K128" s="12" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="L128" s="12" t="s">
         <v>452</v>
       </c>
       <c r="M128" s="20" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="N128" s="2"/>
       <c r="O128" s="2"/>
@@ -8661,16 +8664,16 @@
       <c r="B129" s="2"/>
       <c r="C129" s="2"/>
       <c r="D129" s="1" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="E129" s="9" t="s">
+        <v>612</v>
+      </c>
+      <c r="F129" t="s">
+        <v>612</v>
+      </c>
+      <c r="G129" s="12" t="s">
         <v>613</v>
-      </c>
-      <c r="F129" t="s">
-        <v>613</v>
-      </c>
-      <c r="G129" s="12" t="s">
-        <v>614</v>
       </c>
       <c r="H129" s="12" t="s">
         <v>519</v>
@@ -8682,13 +8685,13 @@
         <v>30</v>
       </c>
       <c r="K129" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L129" s="12" t="s">
         <v>452</v>
       </c>
       <c r="M129" s="20" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="N129" s="2"/>
       <c r="O129" s="2"/>
@@ -8714,16 +8717,16 @@
       <c r="B130" s="2"/>
       <c r="C130" s="2"/>
       <c r="D130" s="1" t="s">
+        <v>615</v>
+      </c>
+      <c r="E130" t="s">
         <v>616</v>
       </c>
-      <c r="E130" t="s">
+      <c r="F130" t="s">
+        <v>616</v>
+      </c>
+      <c r="G130" s="12" t="s">
         <v>617</v>
-      </c>
-      <c r="F130" t="s">
-        <v>617</v>
-      </c>
-      <c r="G130" s="12" t="s">
-        <v>618</v>
       </c>
       <c r="H130" s="12" t="s">
         <v>519</v>
@@ -8735,13 +8738,13 @@
         <v>30</v>
       </c>
       <c r="K130" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L130" s="12" t="s">
         <v>452</v>
       </c>
       <c r="M130" s="20" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="N130" s="2"/>
       <c r="O130" s="2"/>
@@ -8767,16 +8770,16 @@
       <c r="B131" s="2"/>
       <c r="C131" s="2"/>
       <c r="D131" s="1" t="s">
+        <v>619</v>
+      </c>
+      <c r="E131" s="9" t="s">
+        <v>621</v>
+      </c>
+      <c r="F131" s="12" t="s">
         <v>620</v>
       </c>
-      <c r="E131" s="9" t="s">
-        <v>622</v>
-      </c>
-      <c r="F131" s="12" t="s">
-        <v>621</v>
-      </c>
       <c r="G131" s="12" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="H131" s="12" t="s">
         <v>519</v>
@@ -8788,13 +8791,13 @@
         <v>30</v>
       </c>
       <c r="K131" s="12" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="L131" s="12" t="s">
         <v>452</v>
       </c>
       <c r="M131" s="10" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="N131" s="2"/>
       <c r="O131" s="2"/>
@@ -8820,13 +8823,13 @@
       <c r="B132" s="2"/>
       <c r="C132" s="2"/>
       <c r="D132" s="1" t="s">
+        <v>623</v>
+      </c>
+      <c r="E132" s="9" t="s">
         <v>624</v>
       </c>
-      <c r="E132" s="9" t="s">
-        <v>625</v>
-      </c>
       <c r="F132" s="12" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="G132" s="12" t="s">
         <v>177</v>
@@ -8841,13 +8844,13 @@
         <v>30</v>
       </c>
       <c r="K132" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L132" s="12" t="s">
         <v>452</v>
       </c>
       <c r="M132" s="20" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="N132" s="2"/>
       <c r="O132" s="2"/>
@@ -8873,13 +8876,13 @@
       <c r="B133" s="2"/>
       <c r="C133" s="2"/>
       <c r="D133" s="1" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="E133" s="9" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="F133" s="12" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="G133" s="12" t="s">
         <v>177</v>
@@ -8894,13 +8897,13 @@
         <v>30</v>
       </c>
       <c r="K133" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L133" s="12" t="s">
         <v>452</v>
       </c>
       <c r="M133" s="10" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="N133" s="2"/>
       <c r="O133" s="2"/>
@@ -8926,13 +8929,13 @@
       <c r="B134" s="2"/>
       <c r="C134" s="2"/>
       <c r="D134" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="E134" s="9" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="F134" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="G134" s="12" t="s">
         <v>89</v>
@@ -8947,13 +8950,13 @@
         <v>30</v>
       </c>
       <c r="K134" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L134" s="12" t="s">
         <v>452</v>
       </c>
       <c r="M134" s="10" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="N134" s="2"/>
       <c r="O134" s="2"/>
@@ -8979,16 +8982,16 @@
       <c r="B135" s="2"/>
       <c r="C135" s="2"/>
       <c r="D135" s="1" t="s">
+        <v>630</v>
+      </c>
+      <c r="E135" s="9" t="s">
         <v>631</v>
       </c>
-      <c r="E135" s="9" t="s">
+      <c r="F135" s="12" t="s">
         <v>632</v>
       </c>
-      <c r="F135" s="12" t="s">
+      <c r="G135" s="12" t="s">
         <v>633</v>
-      </c>
-      <c r="G135" s="12" t="s">
-        <v>634</v>
       </c>
       <c r="H135" s="12" t="s">
         <v>519</v>
@@ -9000,16 +9003,16 @@
         <v>30</v>
       </c>
       <c r="K135" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L135" s="12" t="s">
         <v>452</v>
       </c>
       <c r="M135" s="20" t="s">
+        <v>634</v>
+      </c>
+      <c r="N135" s="2" t="s">
         <v>635</v>
-      </c>
-      <c r="N135" s="2" t="s">
-        <v>636</v>
       </c>
       <c r="O135" s="2"/>
       <c r="P135" s="2"/>
@@ -9037,7 +9040,7 @@
         <v>486</v>
       </c>
       <c r="E136" s="9" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F136" s="12" t="s">
         <v>487</v>
@@ -9055,7 +9058,7 @@
         <v>98</v>
       </c>
       <c r="K136" s="12" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="L136" s="12" t="s">
         <v>490</v>
@@ -9090,7 +9093,7 @@
         <v>491</v>
       </c>
       <c r="E137" s="9" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="F137" s="12" t="s">
         <v>492</v>
@@ -9108,13 +9111,13 @@
         <v>11</v>
       </c>
       <c r="K137" s="12" t="s">
-        <v>572</v>
+        <v>650</v>
       </c>
       <c r="L137" s="12" t="s">
         <v>494</v>
       </c>
-      <c r="M137" s="12" t="s">
-        <v>541</v>
+      <c r="M137" s="20" t="s">
+        <v>651</v>
       </c>
       <c r="N137" s="2"/>
       <c r="O137" s="2"/>
@@ -9161,7 +9164,7 @@
         <v>98</v>
       </c>
       <c r="K138" s="12" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="L138" s="12" t="s">
         <v>500</v>
@@ -9214,7 +9217,7 @@
         <v>11</v>
       </c>
       <c r="K139" s="12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L139" s="12" t="s">
         <v>500</v>
@@ -9267,7 +9270,7 @@
         <v>11</v>
       </c>
       <c r="K140" s="12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L140" s="12" t="s">
         <v>513</v>
@@ -9320,7 +9323,7 @@
         <v>11</v>
       </c>
       <c r="K141" s="12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L141" s="12" t="s">
         <v>520</v>
@@ -9373,7 +9376,7 @@
         <v>30</v>
       </c>
       <c r="K142" s="12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="L142" s="12" t="s">
         <v>526</v>
@@ -9426,7 +9429,7 @@
         <v>30</v>
       </c>
       <c r="K143" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="L143" s="12" t="s">
         <v>526</v>
@@ -9479,7 +9482,7 @@
         <v>98</v>
       </c>
       <c r="K144" s="12" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="L144" s="12" t="s">
         <v>526</v>
@@ -38830,6 +38833,14 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="D1:M1"/>
+    <mergeCell ref="D3:M3"/>
+    <mergeCell ref="D21:M21"/>
+    <mergeCell ref="D59:M59"/>
+    <mergeCell ref="D42:M42"/>
+    <mergeCell ref="D35:M35"/>
+    <mergeCell ref="D29:M29"/>
+    <mergeCell ref="D13:M13"/>
     <mergeCell ref="D114:M114"/>
     <mergeCell ref="D119:M119"/>
     <mergeCell ref="D123:M123"/>
@@ -38845,14 +38856,6 @@
     <mergeCell ref="D77:M77"/>
     <mergeCell ref="D75:M75"/>
     <mergeCell ref="D81:M81"/>
-    <mergeCell ref="D1:M1"/>
-    <mergeCell ref="D3:M3"/>
-    <mergeCell ref="D21:M21"/>
-    <mergeCell ref="D59:M59"/>
-    <mergeCell ref="D42:M42"/>
-    <mergeCell ref="D35:M35"/>
-    <mergeCell ref="D29:M29"/>
-    <mergeCell ref="D13:M13"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="M5" r:id="rId1"/>
@@ -38948,8 +38951,9 @@
     <hyperlink ref="M130" r:id="rId91"/>
     <hyperlink ref="M132" r:id="rId92"/>
     <hyperlink ref="M135" r:id="rId93"/>
+    <hyperlink ref="M137" r:id="rId94"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId94"/>
+  <legacyDrawing r:id="rId95"/>
 </worksheet>
 </file>
</xml_diff>